<commit_message>
chore(provenance): synchronize manuscript tables, prune advisory clutter, and release v4.39
</commit_message>
<xml_diff>
--- a/thesis_docs/exhibits/ch03_methodology/workbooks/03_Modeling_and_Evaluation.xlsx
+++ b/thesis_docs/exhibits/ch03_methodology/workbooks/03_Modeling_and_Evaluation.xlsx
@@ -1710,7 +1710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -1803,7 +1803,7 @@
       </c>
       <c r="D7" s="18" t="inlineStr">
         <is>
-          <t>Slashed holdout error by 200.9 pax/hr (14.4%) over status-quo scheduling.</t>
+          <t>Slashed holdout error by 91.3 pax/hr (29.1%) over status-quo scheduling (from 313.4 to 222.1 pax/hr).</t>
         </is>
       </c>
     </row>
@@ -1815,17 +1815,22 @@
       </c>
       <c r="B8" s="18" t="inlineStr">
         <is>
-          <t>Fails against naive persistence (MASE = 1.083).</t>
+          <t>Fails against naive persistence (MASE = 0.945 vs Baseline Control MASE = 1.000).</t>
         </is>
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>Significantly outperforms naive persistence (MASE_routine = 0.890).</t>
+          <t>Significantly outperforms naive persistence (MASE_routine = 0.662</t>
         </is>
       </c>
       <c r="D8" s="18" t="inlineStr">
         <is>
-          <t>The Diebold-Mariano test proved statistically significant superiority (DM = 74.25, p &lt; 0.0001).</t>
+          <t>RMSE = 222.1 pax/hr).</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>The Diebold-Mariano test proved statistically significant superiority (DM = 48.72, p &lt; 0.0001).</t>
         </is>
       </c>
     </row>
@@ -1837,17 +1842,17 @@
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>Rigid linear scaling (RMSE = 1,370.3).</t>
+          <t>Preserves stable transfer geometry (RMSE = 326.5 pax/hr; RTR = 1.04).</t>
         </is>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>Physics-based arrival kernel transfers cleanly across layouts.</t>
+          <t>Overfits local terminal layout and innovation feedback (RMSE = 264.3 pax/hr; RTR = 1.19).</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>Maintained lowest absolute zero-shot transfer error (1,162.8 pax/hr, only +7.9% degradation).</t>
+          <t>Model 1 maintained lowest zero-shot transfer degradation (+4.2% RMSE increase and +4.0% DeltaMASE vs Model 3 +19.0% RMSE increase and +21.5% DeltaMASE).</t>
         </is>
       </c>
     </row>

</xml_diff>